<commit_message>
KI-Workshop: Meilenstein-Folie + Fortschritts-Anzeige im MC
- Neue Folie "Vom Buchdruck zur KI" (Zeitstrahl + Adoptions-Tempo) via
  build_meilenstein_folie.py, Stil an Titelfolie angelehnt
- MC-Workshop-Seite: Live-Fortschrittsbalken (GET /api/workshop/fortschritt),
  Helper scripts/ws_fs.py schreibt Status
- Ideensammlung + Auftrag aktualisiert (Themenblock 1 erledigt)
</commit_message>
<xml_diff>
--- a/korrektur/Klasse_9b_WiPo.xlsx
+++ b/korrektur/Klasse_9b_WiPo.xlsx
@@ -97,7 +97,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +144,11 @@
         <fgColor rgb="00FCA5A5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EF4444"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -171,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -234,6 +239,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -651,8 +662,8 @@
           <t>Hoffmann</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n">
-        <v>4</v>
+      <c r="C4" s="24" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -818,7 +829,7 @@
         </is>
       </c>
       <c r="C34" s="12" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>
@@ -1035,14 +1046,14 @@
           <t>Hoffmann</t>
         </is>
       </c>
-      <c r="C3" s="21" t="n">
-        <v>4</v>
+      <c r="C3" s="25" t="n">
+        <v>5</v>
       </c>
       <c r="D3" s="14" t="n"/>
       <c r="E3" s="14" t="n"/>
       <c r="F3" s="14" t="n"/>
       <c r="G3" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
@@ -1326,13 +1337,13 @@
         </is>
       </c>
       <c r="C33" s="18" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
       <c r="F33" s="19" t="n"/>
       <c r="G33" s="12" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>